<commit_message>
Sumas no remunerativas, jornada parcial y aportes Art. 100/101
Validado contra recibos reales de septiembre 2026 (tres empleados, uno a 4 hs):
el motor los reproduce al centavo.

- Escala: columna opcional "No remunerativo" por categoría y vigencia
- Antigüedad y presentismo también sobre la suma no remunerativa
- Asignación extraordinaria no remunerativa por liquidación
- Jornada parcial (horas/8) con obra social y Art. 101 completados a jornada completa
- Aportes Art. 100 y Art. 101 (2% c/u) sobre rem + no rem; se quita la cuota
  sindical "solo afiliados", que no coincide con los recibos reales
- Neto redondeado para arriba al peso
- Recibo con columna No remunerativo

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FTDTDmFZZFvkEzPbBBeoPz
</commit_message>
<xml_diff>
--- a/ejemplos/escala_comercio_ejemplo.xlsx
+++ b/ejemplos/escala_comercio_ejemplo.xlsx
@@ -429,12 +429,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,6 +454,11 @@
           <t>Vigencia desde</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>No remunerativo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,10 +467,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1050000</v>
+        <v>1180000</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="3">
@@ -474,10 +483,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1065750</v>
+        <v>1185900</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="4">
@@ -487,10 +499,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1081736.25</v>
+        <v>1191829.5</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="5">
@@ -500,10 +515,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1097962.29</v>
+        <v>1197788.65</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="6">
@@ -513,10 +531,13 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1114431.73</v>
+        <v>1203777.59</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="7">
@@ -526,10 +547,13 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1131148.2</v>
+        <v>1209796.48</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="8">
@@ -539,10 +563,13 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1148115.43</v>
+        <v>1215845.46</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="9">
@@ -552,10 +579,13 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1165337.16</v>
+        <v>1221924.69</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="10">
@@ -565,10 +595,13 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1182817.22</v>
+        <v>1228034.31</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="11">
@@ -578,10 +611,13 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>1200559.47</v>
+        <v>1234174.48</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="12">
@@ -591,10 +627,13 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1218567.87</v>
+        <v>1240345.36</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="13">
@@ -604,10 +643,13 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1236846.38</v>
+        <v>1246547.08</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="14">
@@ -617,10 +659,13 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1255399.08</v>
+        <v>1252779.82</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="15">
@@ -630,10 +675,13 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>1274230.07</v>
+        <v>1209365</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="16">
@@ -643,10 +691,13 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1293343.52</v>
+        <v>1265338.94</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="17">
@@ -656,10 +707,13 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>1312743.67</v>
+        <v>1271665.63</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="18">
@@ -669,10 +723,13 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1332434.83</v>
+        <v>1278023.96</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="19">
@@ -682,10 +739,13 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1352421.35</v>
+        <v>1284414.08</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="20">
@@ -695,10 +755,13 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1372707.67</v>
+        <v>1290836.15</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="21">
@@ -708,10 +771,13 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1393298.28</v>
+        <v>1297290.33</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="22">
@@ -721,10 +787,13 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>1414197.76</v>
+        <v>1303776.78</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>46204</v>
+        <v>46266</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>120000</v>
       </c>
     </row>
   </sheetData>
@@ -738,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -768,12 +837,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Para un acuerdo nuevo, agregá filas con la nueva vigencia; no borres las anteriores.</t>
+          <t>No remunerativo: suma no remunerativa del acuerdo para ese mes y categoría, jornada completa. Vacío = 0.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>Si el acuerdo cambia la suma no remunerativa mes a mes, cargá una fila por mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Para un acuerdo nuevo, agregá filas con la nueva vigencia; no borres las anteriores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Las categorías tienen que coincidir con las del CCT 130/75 listadas en la plantilla.</t>
         </is>

</xml_diff>